<commit_message>
feat(prioridad): prioriza los leads por cantidad, valor y ganancia con aviso inmediato de los ALTA
</commit_message>
<xml_diff>
--- a/chatbot/hoja/pestanas_bot_itswood.xlsx
+++ b/chatbot/hoja/pestanas_bot_itswood.xlsx
@@ -193,7 +193,7 @@
         <t>El bot la crea en PENDIENTE_HUMANO; después la gestiona el equipo.</t>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
+    <comment ref="AD1" authorId="0" shapeId="0">
       <text>
         <t>Columna del equipo: el bot no la escribe.</t>
       </text>
@@ -26124,7 +26124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2000"/>
+  <dimension ref="A1:AD2000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -26152,7 +26152,11 @@
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="15" customWidth="1" min="24" max="24"/>
     <col width="23" customWidth="1" min="25" max="25"/>
-    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="23" customWidth="1" min="27" max="27"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
+    <col width="23" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -26281,7 +26285,27 @@
           <t>puntaje_intencion</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>valor_estimado</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>ganancia_estimada</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>prioridad</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>puntaje_prioridad</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>notas_equipo</t>
         </is>

</xml_diff>

<commit_message>
feat(fidelizacion): agrega segmentos, recomendaciones postventa y exportación de audiencias
</commit_message>
<xml_diff>
--- a/chatbot/hoja/pestanas_bot_itswood.xlsx
+++ b/chatbot/hoja/pestanas_bot_itswood.xlsx
@@ -18,7 +18,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_PRODUCTOS" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_CLIENTES_FUENTE" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_VENTAS" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_CATALOGO" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_FIDELIZACION" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_CATALOGO" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -278,6 +279,21 @@
 </file>
 
 <file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ITS WOOD bot</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional: escribe NO para ocultar el producto al bot.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>ITS WOOD bot</author>
@@ -12801,7 +12817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2000"/>
+  <dimension ref="A1:K2000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -12811,6 +12827,10 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12847,6 +12867,26 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>acepta_marketing</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>segmento</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>pedidos</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>total_comprado</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ultima_compra</t>
         </is>
       </c>
     </row>
@@ -18919,6 +18959,221 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>segmento</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>canal</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mensaje</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>oferta</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>frecuencia_dias</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CORPORATIVO</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>EMAIL + ASESOR POR WHATSAPP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Hola {nombre}, te compartimos el catálogo corporativo de {negocio}. Para tus próximos regalos te recomendamos {producto}. {oferta}. ¿Agendamos una llamada con un asesor?</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Descuento por volumen desde 50 unidades y logo grabado sin costo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WHATSAPP PERSONAL (HUMANO)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Hola {nombre}, eres de nuestros clientes favoritos de {negocio} 🌳 {oferta}. Te separamos {producto} antes que nadie.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Acceso anticipado a la nueva colección y un regalo en tu próximo pedido</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RECURRENTE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PLANTILLA DE WHATSAPP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Hola {nombre}, a quienes compraron lo mismo que tú también les encantó {producto}. {oferta} 👉 {url}</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>10% de descuento en tu siguiente compra</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EMAIL Y WHATSAPP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>¡Gracias por tu compra, {nombre}! ¿Nos dejas una reseña? Como agradecimiento: {oferta}. Te podría gustar {producto}.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Cupón SEGUNDA10 para tu segunda compra</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DORMIDO</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>WHATSAPP CON CUPÓN + RETARGETING EN META ADS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hola {nombre}, te extrañamos en {negocio}. Vuelve con {oferta}: {producto} te está esperando 👉 {url}</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Cupón VUELVE15 por 15 días</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat(campanas): agrega el flujo [9] de campañas de fidelización con vista previa y envío por email
</commit_message>
<xml_diff>
--- a/chatbot/hoja/pestanas_bot_itswood.xlsx
+++ b/chatbot/hoja/pestanas_bot_itswood.xlsx
@@ -19,7 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_CLIENTES_FUENTE" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_VENTAS" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_FIDELIZACION" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_CATALOGO" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_CAMPANAS" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOT_CATALOGO" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -294,6 +295,21 @@
 </file>
 
 <file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ITS WOOD bot</author>
+  </authors>
+  <commentList>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>El bot la crea en PENDIENTE_HUMANO; después la gestiona el equipo.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>ITS WOOD bot</author>
@@ -19179,6 +19195,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>campana_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>segmento</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>cliente_id</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>canal</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>destino</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>asunto</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>mensaje</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>estado</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>detalle</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H2055"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>